<commit_message>
fix(kit-tareas-heladeria): 3 erratas del ES LIVE (pasteurización, mantecadora en vacío, cilindro), sin cambio de versión
5 celdas de texto en 2 xlsx, parcheadas en el XML (inlineStr): estilos, DV, CF, caché y docProps byte a byte.
- 02 «Pasteurización» B13/B14: grasas y emulsionantes ANTES de pasteurizar, «40-50 °C en ascenso» (iban después,
  «en descenso»: entraban crudos en la mezcla ya pasteurizada).
- 05 «Gestión Semanal» B6: fuera el «test de mantecadora en vacío» (los fabricantes lo prohíben): revisión de
  cuchillas, batidor y junta y la temperatura de extracción en la primera tanda.
- 02 «Mantecación» B24 y 05 «Limpieza Semanal» B13: el cilindro no se desmonta, se limpia en su sitio.
Volcado ES antes/después: solo cambian esas 5 celdas. censo-entregables 0 defectos, no-latinos 0. El generador
(scripts/generate-tareas-heladeria.py) lleva los mismos textos. Revisión adversarial F2 de la EN commiteada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas-heladeria/02-partidas-produccion.xlsx
+++ b/astro-site/public/dl/kit-tareas-heladeria/02-partidas-produccion.xlsx
@@ -967,7 +967,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Pasteurizar a 85 °C durante 15 segundos (alta pasteurización)</t>
+          <t>Añadir grasas y emulsionantes al alcanzar 40-50 °C en ascenso</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Añadir grasas y emulsionantes al alcanzar 40-50 °C en descenso</t>
+          <t>Pasteurizar a 85 °C durante 15 segundos (alta pasteurización)</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Limpiar mantecadora: desmontar cuchillas, junta, cilindro</t>
+          <t>Limpiar mantecadora: desmontar cuchillas, batidor y junta; el cilindro se limpia en su sitio</t>
         </is>
       </c>
       <c r="C24" s="15" t="inlineStr">

</xml_diff>